<commit_message>
Fixed addition of co2 transport
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE26"/>
+  <dimension ref="A1:AE32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3157,6 +3157,624 @@
       <c r="AE26" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\20250915104835_carbon_tax_150_el_price_125</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="M27" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="N27" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>706386.4011532156</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" t="n">
+        <v>2.703999996185303</v>
+      </c>
+      <c r="W27" t="n">
+        <v>35319320.05765668</v>
+      </c>
+      <c r="X27" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>3.449618816375732e-06</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_25</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\20260113182242_carbon_tax_50_el_price_25</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="M28" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="N28" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>706386.4011532156</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>1.718999862670898</v>
+      </c>
+      <c r="W28" t="n">
+        <v>35319320.05765668</v>
+      </c>
+      <c r="X28" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>3.449618816375732e-06</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\20260113182423_carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="M29" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="N29" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>706386.4011532156</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" t="n">
+        <v>2.123999834060669</v>
+      </c>
+      <c r="W29" t="n">
+        <v>35319320.05765668</v>
+      </c>
+      <c r="X29" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>3.449618816375732e-06</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_75</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\20260113182642_carbon_tax_50_el_price_75</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="M30" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="N30" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>706386.4011532156</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
+        <v>2.660000085830688</v>
+      </c>
+      <c r="W30" t="n">
+        <v>35319320.05765668</v>
+      </c>
+      <c r="X30" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>3.449618816375732e-06</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_25</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\20260113183214_carbon_tax_50_el_price_25</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="M31" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="N31" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>706386.4011532156</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" t="n">
+        <v>2.210999965667725</v>
+      </c>
+      <c r="W31" t="n">
+        <v>35319320.05765668</v>
+      </c>
+      <c r="X31" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>3.449618816375732e-06</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\20260113183425_carbon_tax_50_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="M32" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="N32" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>706386.4011532066</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>706386.4011532156</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" t="n">
+        <v>3.136999845504761</v>
+      </c>
+      <c r="W32" t="n">
+        <v>35319320.05765668</v>
+      </c>
+      <c r="X32" t="n">
+        <v>35319320.05766013</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>3.449618816375732e-06</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>carbon_tax_50_el_price_75</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\20260113184050_carbon_tax_50_el_price_75</t>
         </is>
       </c>
     </row>

</xml_diff>